<commit_message>
Refine D7 figures to Nature publication standard
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_audit_log.xlsx
@@ -913,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -940,11 +940,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13602</v>
+        <v>14506</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>8ba0309e3568e5c4860a71fb4789cd621cc704b6366b86bd23bd8727b87cc84e</t>
+          <t>ccfbca5b9dd57957714bded6fc9e99e6d502b16e91c7896ad0347d8f3658f0f3</t>
         </is>
       </c>
     </row>
@@ -955,11 +955,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2382</v>
+        <v>3200</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>89d5b54cdb4b970d95acb829f7ddf6eb230b270d6000dd8c87047f29c6f1c3d4</t>
+          <t>a12d21fd62dd04f5d6dcd660f41bde69f941e4f4a9ccf1cda2e1623d61089a32</t>
         </is>
       </c>
     </row>
@@ -970,11 +970,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>49208</v>
+        <v>51706</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>309e462028bd4b6ff796d4c6627f36a4e82d665afe6c29d07dfd70f5866257a1</t>
+          <t>2f1abed0142d2617649cf488d33cfc996ab0cd89c918d15788226139201b978c</t>
         </is>
       </c>
     </row>
@@ -985,11 +985,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>282038</v>
+        <v>315954</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3d4abf7093191a47db0e323225200ccf9f03106afb818dade304137401ebb469</t>
+          <t>b8d6b85f4de5f3b1fa8eaf072ceb49e927f0936e248b69ce8363889076a5dfc2</t>
         </is>
       </c>
     </row>
@@ -1000,924 +1000,999 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37998</v>
+        <v>28772</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>bc3f147b7b79ae412151717ff8450396368a89451ae38599788c12fb1ff8d96f</t>
+          <t>a1ad2baf716112cb511807d080f4a6eef164ce779dbdf1736c817fbf69c8af67</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_2_spatiotemporal.pdf</t>
+          <t>outputs/figures/FigD7_1_framework.tiff</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>68792</v>
+        <v>620316</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0730bb25fb25f32f10f8ca24bbe9ffcb7268dc65daced0447ad91b523fe874b6</t>
+          <t>fa89c5f1fb49f0ad9ee0978df75a4d2aeab0bfb4d14efd1ebc9c6e0c78c44f25</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_2_spatiotemporal.png</t>
+          <t>outputs/figures/FigD7_2_spatiotemporal.pdf</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>345707</v>
+        <v>63355</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>54df2039c1f7089650f77d0290fc425757a27b3fca852bcf4a65fa8e44837889</t>
+          <t>14290cb202b7cfe5dcdca221de89023aabd324fded52f87c207f9173df0784ba</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_2_spatiotemporal.svg</t>
+          <t>outputs/figures/FigD7_2_spatiotemporal.png</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>70324</v>
+        <v>385799</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>d3ad18ca714624bfc20b20ca22f7c5933af77ffa342eb789474953970cd7246d</t>
+          <t>055f03c1decf7348eb20b879356faaadb23329fe9a86f9f1803d8ff3444a4b88</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_3_evidence.pdf</t>
+          <t>outputs/figures/FigD7_2_spatiotemporal.svg</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>54403</v>
+        <v>69127</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>8a9e29f8a55d2c569e2767104100b48bdffd8ac81de2b8012206269c19da90ce</t>
+          <t>7cdf92f33c51439e135456d40a72a2da7dd470ec6d5b25c5e97cca5db13c0915</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_3_evidence.png</t>
+          <t>outputs/figures/FigD7_2_spatiotemporal.tiff</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>573661</v>
+        <v>7350736</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>a2db09eaeb1480d9fb757d780c4447c44585ec534a7eba04524acd5167011179</t>
+          <t>35c45a2caff1b1f979ff182f6e44550a015115a613fa18fbc8dc43ee673ef7b0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_3_evidence.svg</t>
+          <t>outputs/figures/FigD7_3_evidence.pdf</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>55032</v>
+        <v>54046</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ee6adc7047acd4f464465e023c8bbf792a9336a1f710171596a0e4d8fe40856a</t>
+          <t>99086a3dbe481d6a5b71f04626512c9605e69ecab78130371413f7a8317a2dc5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_4_validation.pdf</t>
+          <t>outputs/figures/FigD7_3_evidence.png</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>48000</v>
+        <v>595335</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4a21542da846a97dae48596083568b7709001f9b71e7011787984cd8d3b1ec21</t>
+          <t>7507c754eef39ce1c96afb784a37d58c844b26078acef706bdecf7aad56f5b63</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_4_validation.png</t>
+          <t>outputs/figures/FigD7_3_evidence.svg</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>521976</v>
+        <v>52383</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>fa07824828da0bad99cbbea776dd59a96fb3f486e3805046d64cbb97fdcafe80</t>
+          <t>a67694554c53b927e68a088acd97c1a18ff9e0ac7c22f42621750b28f1be48a9</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_4_validation.svg</t>
+          <t>outputs/figures/FigD7_3_evidence.tiff</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>41913</v>
+        <v>1289062</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7d0ae9c723b16a530e7fc878a0c6b690c1fc620397996152bff9c5f032a28832</t>
+          <t>69331122bd027fd523493fc5a2fd7e5b524ad87963514787a37250ea11d4735d</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_5_governance.pdf</t>
+          <t>outputs/figures/FigD7_4_validation.pdf</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>52504</v>
+        <v>53521</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>08f6f69ee37df189f2200059b0927e8c09e32dbfd789436c3bfff370febc6e32</t>
+          <t>5e5f64c034ddfe8271003b0590f9da48648110e094e4c6cee27fc363e0d2a3ef</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_5_governance.png</t>
+          <t>outputs/figures/FigD7_4_validation.png</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>520537</v>
+        <v>471042</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>f972c07dbc579296ad8a1c8faaadf0c67943bb380e333121fab6f37b61c66031</t>
+          <t>8f10fe158f6cd498110b4c737a70887913c8e64f93d6cb294ee171f44c5f117c</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>outputs/figures/FigD7_5_governance.svg</t>
+          <t>outputs/figures/FigD7_4_validation.svg</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>45570</v>
+        <v>45044</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>cfd99844a2db4600ea81cf29216573b90004f7172ef34dc1c0f1f620807b5146</t>
+          <t>7bb965b089228a9e4050712be175038b1f26004b9d9ceda4e5c239e754c48dff</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>outputs/local/D7_ablation_redundancy.xlsx</t>
+          <t>outputs/figures/FigD7_4_validation.tiff</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>9861</v>
+        <v>985686</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>a96ebb1d62b794f709fcb8d8a048711bbf58cb80d202b2f26e46f5a783eab8a4</t>
+          <t>bbd879ad74d9a5a8172f0b578a4cb0aedc7262e4dd299d5bf3d37690c8989576</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>outputs/local/D7_audit_log.xlsx</t>
+          <t>outputs/figures/FigD7_5_governance.pdf</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>84792</v>
+        <v>51533</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0f135dac17109aa947fa780339d01da2bf72f450d246f43bdfd6b8ba5ae5108f</t>
+          <t>e638c86ce4a5e9ea7bc2c40a96d2ada79b5c66d9374182e791908977d68b07db</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>outputs/local/D7_case_study_exports.xlsx</t>
+          <t>outputs/figures/FigD7_5_governance.png</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>44230</v>
+        <v>470003</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>3671e79cdc4ed4f640a63b5e65969ff7d7b86037c0c36f4a98615924e2e5eed8</t>
+          <t>262b314c910ea2fdb5ea220cd8880ed324b2594a148643235c064d1b562bf250</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>outputs/local/D7_d6_interface.schema.json</t>
+          <t>outputs/figures/FigD7_5_governance.svg</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>546</v>
+        <v>39607</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>edc1c46088deb146df6c97efa7a124997e08ceeb0179f609e5e6705908349ba1</t>
+          <t>d824042d7f7929fd2841ba2cb1ca259bb374289b7a3770f2865327013d4a4c9f</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>outputs/local/D7_edge_profile_summary.xlsx</t>
+          <t>outputs/figures/FigD7_5_governance.tiff</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>30812</v>
+        <v>993666</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0fab41c05d378d234a33f938f8f81748ba24795b12b908c9a8c310206aea5599</t>
+          <t>a8124854db0f374f5388dad55aafb6d19f994ab04184b787c0294735f5455c70</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>outputs/local/D7_event_windows.parquet</t>
+          <t>outputs/local/D7_ablation_redundancy.xlsx</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>70845</v>
+        <v>9861</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>7fc6239ad5b77da66e04d4abcce8a20621fc7ce111915cfb5fe50cfb7de4f830</t>
+          <t>a96ebb1d62b794f709fcb8d8a048711bbf58cb80d202b2f26e46f5a783eab8a4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>outputs/local/D7_event_windows.xlsx</t>
+          <t>outputs/local/D7_audit_log.xlsx</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>126116</v>
+        <v>85126</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0aa4b388d803cb087e7d0bf36829314f997dac14d39f57ab92a0b23362f352d7</t>
+          <t>6996b7b8916d73721583227be6ee6c2c448e44598f7d0082436e918a724fde97</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>outputs/local/D7_main_scores_hourly.parquet</t>
+          <t>outputs/local/D7_case_study_exports.xlsx</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>9816871</v>
+        <v>44230</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0f64524fc8b543be2d5da33901c5c7b1e3ca6655841c4489bbebb660481123cf</t>
+          <t>3671e79cdc4ed4f640a63b5e65969ff7d7b86037c0c36f4a98615924e2e5eed8</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>outputs/local/D7_main_scores_hourly.xlsx</t>
+          <t>outputs/local/D7_d6_interface.schema.json</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>32383539</v>
+        <v>546</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>c1642b17924fb22d3165f17b107f0615a039ce3fda940e4952545eb4013b555c</t>
+          <t>edc1c46088deb146df6c97efa7a124997e08ceeb0179f609e5e6705908349ba1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>outputs/local/D7_mapping_params.xlsx</t>
+          <t>outputs/local/D7_edge_profile_summary.xlsx</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>20273</v>
+        <v>30812</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>46d7355c413cdfb67a494f2fefb51c4f333dbaa5c413a1bc0e2ff802341c0d35</t>
+          <t>0fab41c05d378d234a33f938f8f81748ba24795b12b908c9a8c310206aea5599</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>outputs/local/D7_multiscale_aggregates.xlsx</t>
+          <t>outputs/local/D7_event_windows.parquet</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>929096</v>
+        <v>70845</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1c61b75561978916b83b9ca03f6485e17890d9719f3ad5d8e5bac22b7866266e</t>
+          <t>7fc6239ad5b77da66e04d4abcce8a20621fc7ce111915cfb5fe50cfb7de4f830</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>outputs/local/D7_reference_window_library.parquet</t>
+          <t>outputs/local/D7_event_windows.xlsx</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>63489</v>
+        <v>126116</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>79a8bb6da54a371c394721ec37fe43b47fdcfe603047396fd2a609f76fcf90a2</t>
+          <t>0aa4b388d803cb087e7d0bf36829314f997dac14d39f57ab92a0b23362f352d7</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>outputs/local/D7_reference_window_library.xlsx</t>
+          <t>outputs/local/D7_main_scores_hourly.parquet</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>217159</v>
+        <v>9816871</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>5ab6dab08111d83cc882f14cde37e8a44cd4fe791d33d2bdc31149c4b7a5c84e</t>
+          <t>0f64524fc8b543be2d5da33901c5c7b1e3ca6655841c4489bbebb660481123cf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>outputs/local/D7_regime_state.parquet</t>
+          <t>outputs/local/D7_main_scores_hourly.xlsx</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>30965123</v>
+        <v>32383539</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>4bcc9fc4963a076ac3367f66933906514d3059b9558fe7ecf35112a210b0975b</t>
+          <t>c1642b17924fb22d3165f17b107f0615a039ce3fda940e4952545eb4013b555c</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>outputs/local/D7_regime_state.xlsx</t>
+          <t>outputs/local/D7_mapping_params.xlsx</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>86555483</v>
+        <v>20273</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2b6a21f2bcbb3e0bc98224b4a0bef0fd88fa6241bf0076779a2a461514578a39</t>
+          <t>46d7355c413cdfb67a494f2fefb51c4f333dbaa5c413a1bc0e2ff802341c0d35</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>outputs/local/D7_sensor_influence.parquet</t>
+          <t>outputs/local/D7_multiscale_aggregates.xlsx</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>5711635</v>
+        <v>929096</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>551b51782ab00fa2a45ce788c736a3a786f5e98bd0decf442386e98c10ceeca8</t>
+          <t>1c61b75561978916b83b9ca03f6485e17890d9719f3ad5d8e5bac22b7866266e</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>outputs/local/D7_sensor_influence.xlsx</t>
+          <t>outputs/local/D7_reference_window_library.parquet</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>12919122</v>
+        <v>63489</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>6f0b729daaad6291eb28e16cb5a3cd7bb04359b7133247073d7d2cedb2fae802</t>
+          <t>79a8bb6da54a371c394721ec37fe43b47fdcfe603047396fd2a609f76fcf90a2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>outputs/local/D7_sensor_profile_summary.xlsx</t>
+          <t>outputs/local/D7_reference_window_library.xlsx</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>7506</v>
+        <v>217159</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>cc2bf6813e78c833ef9761874514b5bbb77d204df7ebe65ce4fad898cbc22c01</t>
+          <t>5ab6dab08111d83cc882f14cde37e8a44cd4fe791d33d2bdc31149c4b7a5c84e</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>outputs/local/D7_spatial_evidence.parquet</t>
+          <t>outputs/local/D7_regime_state.parquet</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>6696159</v>
+        <v>30965123</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>b0035a5ff086111cc5d18c78e1ea383a4aa71bb395b4a0487048293dd9b83eb4</t>
+          <t>4bcc9fc4963a076ac3367f66933906514d3059b9558fe7ecf35112a210b0975b</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>outputs/local/D7_spatial_evidence.xlsx</t>
+          <t>outputs/local/D7_regime_state.xlsx</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>16026614</v>
+        <v>86555483</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>fcbc3809f84eff23290f3b39ef1bfd7715c352e7f9d8297a8618ac3746c08ec2</t>
+          <t>2b6a21f2bcbb3e0bc98224b4a0bef0fd88fa6241bf0076779a2a461514578a39</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>outputs/local/D7_spatial_templates.template_bundle.json</t>
+          <t>outputs/local/D7_sensor_influence.parquet</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>452892</v>
+        <v>5711635</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>05166df2a55b4827a95a3755df1e38f085f99c80f71d5099f099774d6db2646c</t>
+          <t>551b51782ab00fa2a45ce788c736a3a786f5e98bd0decf442386e98c10ceeca8</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>outputs/local/D7_spatial_templates.xlsx</t>
+          <t>outputs/local/D7_sensor_influence.xlsx</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>186908</v>
+        <v>12919122</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>89963486def67ccf2bcf0b43cd3190b24fb1ecdb7fc77940b4f679cafa1e2842</t>
+          <t>6f0b729daaad6291eb28e16cb5a3cd7bb04359b7133247073d7d2cedb2fae802</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>outputs/local/D7_support_assessment.parquet</t>
+          <t>outputs/local/D7_sensor_profile_summary.xlsx</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>28123</v>
+        <v>7506</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>833ffa282f79fca883fa791c7ccd9a8113af3e3237190128d7d8ee8f981fdb9b</t>
+          <t>cc2bf6813e78c833ef9761874514b5bbb77d204df7ebe65ce4fad898cbc22c01</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>outputs/local/D7_support_assessment.xlsx</t>
+          <t>outputs/local/D7_spatial_evidence.parquet</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>17720</v>
+        <v>6696159</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ccceea1092f3c097c044bf903f72e667fec5c14b06ef0a52a827d33e4f2f0d24</t>
+          <t>b0035a5ff086111cc5d18c78e1ea383a4aa71bb395b4a0487048293dd9b83eb4</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>outputs/local/D7_topology_drift_alerts.parquet</t>
+          <t>outputs/local/D7_spatial_evidence.xlsx</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>10784</v>
+        <v>16026614</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>3b6fc36c522d6fa0eeaba6ba5408caa8079958dc899eeaf353cf437163104100</t>
+          <t>fcbc3809f84eff23290f3b39ef1bfd7715c352e7f9d8297a8618ac3746c08ec2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>outputs/local/D7_topology_drift_alerts.xlsx</t>
+          <t>outputs/local/D7_spatial_templates.template_bundle.json</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>9949</v>
+        <v>452892</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>6b4068d8791367701a84a8befe574e597e7e5c9ad33c108c23c894537e5f4334</t>
+          <t>05166df2a55b4827a95a3755df1e38f085f99c80f71d5099f099774d6db2646c</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>outputs/local/D7_topology_registry.json</t>
+          <t>outputs/local/D7_spatial_templates.xlsx</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>10933</v>
+        <v>186908</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>f85b868e9941538c8da10ae2dbd4f0c0aa4a9f2f784656a1c9fd925ca2a40d08</t>
+          <t>89963486def67ccf2bcf0b43cd3190b24fb1ecdb7fc77940b4f679cafa1e2842</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>outputs/local/D7_topology_registry.schema.json</t>
+          <t>outputs/local/D7_support_assessment.parquet</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>715</v>
+        <v>28123</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>126497fdca42ce676bedc4f83055a445039233d3f6b8b5d056b06e65eee48e37</t>
+          <t>833ffa282f79fca883fa791c7ccd9a8113af3e3237190128d7d8ee8f981fdb9b</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>outputs/local/D7_topology_registry.xlsx</t>
+          <t>outputs/local/D7_support_assessment.xlsx</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>9980</v>
+        <v>17720</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>d287e3075a0d9258964a343239adc2b3df2b3eb27579abdba1a86f80a20ebd8a</t>
+          <t>ccceea1092f3c097c044bf903f72e667fec5c14b06ef0a52a827d33e4f2f0d24</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>outputs/local/D7_topology_registry.yaml</t>
+          <t>outputs/local/D7_topology_drift_alerts.parquet</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2508</v>
+        <v>10784</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>5855cf2bb6d4f570d9d469ee541107ff429951b08067298e78fb1a0f7296c8d0</t>
+          <t>3b6fc36c522d6fa0eeaba6ba5408caa8079958dc899eeaf353cf437163104100</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>outputs/local/D7_validation_results.xlsx</t>
+          <t>outputs/local/D7_topology_drift_alerts.xlsx</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>30224</v>
+        <v>9949</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>31db2243406ef1166aee95f61af52402025d51ef5c1136b9f38d98e68f74dd1b</t>
+          <t>6b4068d8791367701a84a8befe574e597e7e5c9ad33c108c23c894537e5f4334</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>outputs/local/D7_zone_consensus.parquet</t>
+          <t>outputs/local/D7_topology_registry.json</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1208845</v>
+        <v>10933</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>74f38faeaf6b9dd523e4f1196ec07221ad359167e0f8dd6348696aac3ae64127</t>
+          <t>f85b868e9941538c8da10ae2dbd4f0c0aa4a9f2f784656a1c9fd925ca2a40d08</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>outputs/local/D7_zone_consensus.xlsx</t>
+          <t>outputs/local/D7_topology_registry.schema.json</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>4773714</v>
+        <v>715</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>87f355c32b07e5cfb17dcbd9604b9aad3f2b98a2708dbc05132d171b6f17f6c5</t>
+          <t>126497fdca42ce676bedc4f83055a445039233d3f6b8b5d056b06e65eee48e37</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D7_plot_data.csv</t>
+          <t>outputs/local/D7_topology_registry.xlsx</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>5165042</v>
+        <v>9980</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>9cf0b67991f5d9d0aa07c005f1ae20e2d29f9bc7003918cb82874aed80d00885</t>
+          <t>d287e3075a0d9258964a343239adc2b3df2b3eb27579abdba1a86f80a20ebd8a</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D7_plot_data.parquet</t>
+          <t>outputs/local/D7_topology_registry.yaml</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>180365</v>
+        <v>2508</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>07c67efc62194833637deea96361abe3a4905f17786446eeaffb1fbc60d703a3</t>
+          <t>5855cf2bb6d4f570d9d469ee541107ff429951b08067298e78fb1a0f7296c8d0</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>outputs/plot_data/D7_plot_data_manifest.json</t>
+          <t>outputs/local/D7_validation_results.xlsx</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>519</v>
+        <v>30224</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>41e144f18ead76df5b4a82453258b04985950e871e4bf2553a18f41cc70b2632</t>
+          <t>31db2243406ef1166aee95f61af52402025d51ef5c1136b9f38d98e68f74dd1b</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>outputs/reports/D7_EXPERT_REPORT_v2.1.docx</t>
+          <t>outputs/local/D7_zone_consensus.parquet</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1930105</v>
+        <v>1208845</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>de5bff6d2b0b19d12b5b87eb0d11bb4e7da1bf313af43764faeaa5e7e80a5f50</t>
+          <t>74f38faeaf6b9dd523e4f1196ec07221ad359167e0f8dd6348696aac3ae64127</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>outputs/reports/D7_EXPERT_REPORT_v2.1.md</t>
+          <t>outputs/local/D7_zone_consensus.xlsx</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>6008</v>
+        <v>4773714</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>7b33f201e4a4024c5f46152da4b0eeb0eb150f15f396087a3eacf4735d7173af</t>
+          <t>87f355c32b07e5cfb17dcbd9604b9aad3f2b98a2708dbc05132d171b6f17f6c5</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>outputs/reports/D7_FIGURE_CAPTIONS_v2.1.md</t>
+          <t>outputs/plot_data/D7_plot_data.csv</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>2022</v>
+        <v>27713153</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>79c715bb3df74ec90b1816f911bf2a88f36fa7ad71e4f6262b6d3df8b470469e</t>
+          <t>ee688d5969652f0a4d9a045229bf4fa7e4d92694b7630f31437e4fc55faab97b</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>outputs/reports/D7_PROJECT_DIRECTORY_GUIDE_v2.1.docx</t>
+          <t>outputs/plot_data/D7_plot_data.parquet</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>40298</v>
+        <v>896956</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2cce4bf06a2f8825476b1c551a897e1047e1f5a67e354ba330ecaa5f423b92b2</t>
+          <t>9740bc0a48d5679b2e03c791b49e34c0adfce06f85abb252ad26eea128703526</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>outputs/reports/D7_PROJECT_DIRECTORY_GUIDE_v2.1.md</t>
+          <t>outputs/plot_data/D7_plot_data_manifest.json</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>4870</v>
+        <v>856</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>269d82cbb7dc64ca7fa0efb8c86535600cf8da72f3aae06aa448794195637a82</t>
+          <t>2da736bd764b8c6ca819aa256a4fa917ff90edccce5d18820ffc6c43d020288c</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D7_sensitivity_manifest.json</t>
+          <t>outputs/reports/D7_EXPERT_REPORT_v2.1.docx</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1400</v>
+        <v>1994234</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>bd0d7a20ba97af03e87f2c66570ce6fb67b1468394aa3401b9ee8f51c6cea26d</t>
+          <t>53cfd78c1ad0d2946b8e361958747016936cc7ddb38bbf01a840c1f9477e7a99</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D7_shadow_scores.parquet</t>
+          <t>outputs/reports/D7_EXPERT_REPORT_v2.1.md</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2966985</v>
+        <v>6202</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>5a20c2b223c25f33756c868fa2eebd0d4f25b0510c46cc99d9612d665abad6b9</t>
+          <t>0e7db5c3ac36ec1b0305bd44d92caaafb0adda60865953bebe24a07944e4273f</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D7_shadow_scores.xlsx</t>
+          <t>outputs/reports/D7_FIGURE_CAPTIONS_v2.1.md</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>10049007</v>
+        <v>2263</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>eac37ae348e7dbb9c062331975a9631d1c1369a68e7c45f3ef30bed775a59c0c</t>
+          <t>4ae54945b07f517736422b6ecd412dd68085f9b393e064e347e8662d989f8df0</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D7_shadow_template_shift.xlsx</t>
+          <t>outputs/reports/D7_PROJECT_DIRECTORY_GUIDE_v2.1.docx</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>41716</v>
+        <v>40309</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>6e4f528897face976d57525a071f3c79a9062c1c23d74509d16362948ff5962d</t>
+          <t>83c6b5df38dc0d98ed5b89c96c5d696056887286b5629009b9601b906dcdcc8a</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>outputs/sensitivity/D7_track_invariance.xlsx</t>
+          <t>outputs/reports/D7_PROJECT_DIRECTORY_GUIDE_v2.1.md</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>14475</v>
+        <v>4887</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>a0dc72455ca2838b4628b24794b545403d21172f59cb5c277a01127d49383410</t>
+          <t>5add68cc0d5f038586d648929100385fbc0cc70af62fe2fb9e15f6145d01e00b</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>outputs/shadow_v2/D7_graph_structure_learning_shadow.parquet</t>
+          <t>outputs/sensitivity/D7_sensitivity_manifest.json</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>9348</v>
+        <v>1400</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>d5c5d09e445021f08ef4bc32d14aef2b7e28fb52ce807395176d750c987ad0da</t>
+          <t>bd0d7a20ba97af03e87f2c66570ce6fb67b1468394aa3401b9ee8f51c6cea26d</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>outputs/shadow_v2/D7_graph_structure_learning_shadow.xlsx</t>
+          <t>outputs/sensitivity/D7_shadow_scores.parquet</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>8313</v>
+        <v>2966985</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>5128724d8e273420d1f87f8561bbe4699dd9f949898f51583947b0cf153aff72</t>
+          <t>5a20c2b223c25f33756c868fa2eebd0d4f25b0510c46cc99d9612d665abad6b9</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>outputs/sensitivity/D7_shadow_scores.xlsx</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>10049007</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>eac37ae348e7dbb9c062331975a9631d1c1369a68e7c45f3ef30bed775a59c0c</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D7_shadow_template_shift.xlsx</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>41716</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>6e4f528897face976d57525a071f3c79a9062c1c23d74509d16362948ff5962d</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>outputs/sensitivity/D7_track_invariance.xlsx</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>14475</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>a0dc72455ca2838b4628b24794b545403d21172f59cb5c277a01127d49383410</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>outputs/shadow_v2/D7_graph_structure_learning_shadow.parquet</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>9348</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>d5c5d09e445021f08ef4bc32d14aef2b7e28fb52ce807395176d750c987ad0da</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>outputs/shadow_v2/D7_graph_structure_learning_shadow.xlsx</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>8313</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>5128724d8e273420d1f87f8561bbe4699dd9f949898f51583947b0cf153aff72</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
           <t>outputs/shadow_v2/D7_shadow_v2_manifest.json</t>
         </is>
       </c>
-      <c r="B67" t="n">
+      <c r="B72" t="n">
         <v>263</v>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>fa05e2d31b9b363ca7ed9b5a4cd6eec8f44388bfbf052225243ddde2329ffeed</t>
         </is>

</xml_diff>

<commit_message>
Remove redundant ticks from D7 Figure 2a
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_audit_log.xlsx
@@ -944,7 +944,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ccfbca5b9dd57957714bded6fc9e99e6d502b16e91c7896ad0347d8f3658f0f3</t>
+          <t>c92691d09c8deddf3657ef19e4277dde9da33360004b4c7f89dff5297a41448f</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>a12d21fd62dd04f5d6dcd660f41bde69f941e4f4a9ccf1cda2e1623d61089a32</t>
+          <t>03ae1c18875a33d03f88e9cfe97858065bd07d68bda4bdfde2fd69307a5c0a92</t>
         </is>
       </c>
     </row>
@@ -1030,11 +1030,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>63355</v>
+        <v>63169</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14290cb202b7cfe5dcdca221de89023aabd324fded52f87c207f9173df0784ba</t>
+          <t>600293b719f0a5b1485fc0c89f76b10ce921bece0ac37398515f70b6ac31aecf</t>
         </is>
       </c>
     </row>
@@ -1045,11 +1045,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>385799</v>
+        <v>384819</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>055f03c1decf7348eb20b879356faaadb23329fe9a86f9f1803d8ff3444a4b88</t>
+          <t>7913a3fe1686e1136aa2d2deaa65649217622f377dbc3a1f47d74d0f9c8bc8d9</t>
         </is>
       </c>
     </row>
@@ -1060,11 +1060,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>69127</v>
+        <v>65364</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>7cdf92f33c51439e135456d40a72a2da7dd470ec6d5b25c5e97cca5db13c0915</t>
+          <t>adc3a2ec9c781e2b665190d3c117c564c6dc885ff0365e395a74dfa42bc1ef7f</t>
         </is>
       </c>
     </row>
@@ -1075,11 +1075,11 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7350736</v>
+        <v>7351238</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>35c45a2caff1b1f979ff182f6e44550a015115a613fa18fbc8dc43ee673ef7b0</t>
+          <t>7c5fceec041a4f4d32d5dd54495248b5982c7eaa3c6099f6f86048c9c8d10f82</t>
         </is>
       </c>
     </row>
@@ -1285,11 +1285,11 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>85126</v>
+        <v>85117</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>6996b7b8916d73721583227be6ee6c2c448e44598f7d0082436e918a724fde97</t>
+          <t>b676e4cb2f4f0f6fc5ebbc73787305f7b5beb3121547a89d057d1aaf41758b88</t>
         </is>
       </c>
     </row>
@@ -1810,11 +1810,11 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1994234</v>
+        <v>1992957</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>53cfd78c1ad0d2946b8e361958747016936cc7ddb38bbf01a840c1f9477e7a99</t>
+          <t>ea11e3ada916315ff77216fda15c41b1ae7a9e28164122ca70ce2ce74d7760a1</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0e7db5c3ac36ec1b0305bd44d92caaafb0adda60865953bebe24a07944e4273f</t>
+          <t>78680b1c183f0ea61d4715b9ecd7f98962e154d6bc8ba9595165f07fa15e10fd</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>83c6b5df38dc0d98ed5b89c96c5d696056887286b5629009b9601b906dcdcc8a</t>
+          <t>ce9bb9d4e988b8441420bb1da589e5c35a78bc154dfcd4ad7981a8d0987856b9</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>5add68cc0d5f038586d648929100385fbc0cc70af62fe2fb9e15f6145d01e00b</t>
+          <t>034547f8813a00d410b11d12a37133812ae541138500c7e0bd68d32779d09059</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Standardize publication figures and audit freshness
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_audit_log.xlsx
+++ b/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_audit_log.xlsx
@@ -944,7 +944,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>bd4643d83c7adc995f443d166b7049c389811d775b9dd23f2f021e9156372353</t>
+          <t>c093078b779e0f2570dfc7e8d69c46e6b1be4194f02f377f88f332b781db3709</t>
         </is>
       </c>
     </row>
@@ -955,11 +955,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2382</v>
+        <v>2381</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>e6a4df553688a6a6c3c62afe49e80e7b4d56575913e55f548409ea06f11d3f3f</t>
+          <t>25007a8e5c437cf6a1ce97dbc5d58b42add2d71190e937cde29df3cfa3c6dc77</t>
         </is>
       </c>
     </row>
@@ -970,11 +970,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>49208</v>
+        <v>49360</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>d9a32f4c45fbc37a977d3aa6471439958b9b96dfda833847f6f873654a442521</t>
+          <t>28d38d009df41c8b295fa74488fd90290a095f5b8d2494def28224171304fa6f</t>
         </is>
       </c>
     </row>
@@ -985,11 +985,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>282038</v>
+        <v>276723</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3d4abf7093191a47db0e323225200ccf9f03106afb818dade304137401ebb469</t>
+          <t>b6b62dafe200e9be8de90d6f916cb70e0659ec43063979047b38d935558f35f5</t>
         </is>
       </c>
     </row>
@@ -1000,11 +1000,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37998</v>
+        <v>38538</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3ea5adbd3e99d038c5cee9205769a9667889db607329b3d207474ca7118ebc7f</t>
+          <t>4bdfb2b07797bd1c80841e2a6dc8009e41b8a2e8687905dd1e36512eaa745bfd</t>
         </is>
       </c>
     </row>
@@ -1015,11 +1015,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>68792</v>
+        <v>57645</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0c2c1f35a5c2aae8806f5e894ae7b33195c9c97a3e6e50597f0a8f67488022f0</t>
+          <t>1e59e451fd53c72ee0cf850fdcca5ce1b4cca0775b44ec2a86caf6a31c5e7e15</t>
         </is>
       </c>
     </row>
@@ -1030,11 +1030,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>345707</v>
+        <v>346048</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>54df2039c1f7089650f77d0290fc425757a27b3fca852bcf4a65fa8e44837889</t>
+          <t>65a074c6f602540b91350b99267fee96161df51cc2475fbcc22cbdb337c294e7</t>
         </is>
       </c>
     </row>
@@ -1045,11 +1045,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>70324</v>
+        <v>60008</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>a21ef5ec5f69fa2830f6e45398d60123a35d67350d1e7913dafe545b8f5e6cbf</t>
+          <t>bc3c07ad98e4a7889603e632bec35a61cba6a559054e821c98d70caf09fd06df</t>
         </is>
       </c>
     </row>
@@ -1060,11 +1060,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>54403</v>
+        <v>54621</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9b44a8dbc11b1371807476058aa01ac19a0a5707ea82a93850dbaee3a128b2c9</t>
+          <t>16bc271e20fd4361223d7677b458c909dc551003a39cf1bf7b9680eeed386820</t>
         </is>
       </c>
     </row>
@@ -1075,11 +1075,11 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>573661</v>
+        <v>570148</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>a2db09eaeb1480d9fb757d780c4447c44585ec534a7eba04524acd5167011179</t>
+          <t>946e17bebc7716f5dce800e2d8bca417537abd98e3bc0adb1a8571359e6e6e78</t>
         </is>
       </c>
     </row>
@@ -1090,11 +1090,11 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>55032</v>
+        <v>55621</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0c79b045fb3e9bde63aa590ad4377075ccbe97f8bd9ffd722f39d79d0b479c6b</t>
+          <t>b427b0cad92c5239a18e979ccc97ec47827f9ad71ffedff8c2bf13c2173d0b36</t>
         </is>
       </c>
     </row>
@@ -1105,11 +1105,11 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>48000</v>
+        <v>48157</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>c0edba708a32383e91befd4c55813fba4e2dc4cdbbf4638a4ecd69dfdd7ab40d</t>
+          <t>3cd5b44f2c719147a43d19656eea0145f85a3db14a0f29038e0938b546594977</t>
         </is>
       </c>
     </row>
@@ -1120,11 +1120,11 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>521995</v>
+        <v>520891</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>c3488d51590533f604b71ee41918987c7c7c07604fbf190bec3c653c394db6f4</t>
+          <t>2dc5dd1210cf7323017af5b8f3469aa1e26420a21a8405830c7111673a9be0de</t>
         </is>
       </c>
     </row>
@@ -1135,11 +1135,11 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>41915</v>
+        <v>42706</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>9ef811e36163ea2f00a4eee6fa97549d7cd0c11eddce9ca88f4a6b3b133ed693</t>
+          <t>a2a5f071d9ec7a8f2b91160fef3e7dc5d4d65f6b1ddb11973df353896ea1ef82</t>
         </is>
       </c>
     </row>
@@ -1150,11 +1150,11 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>52504</v>
+        <v>52659</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>da194e7c341735eec0b37c10ede80e76ec1e23af4e651b986987d1e7a13b3780</t>
+          <t>deac4d89588b01514d6d3d3d50717962c352999b89ca59804211b868ae3c8ac4</t>
         </is>
       </c>
     </row>
@@ -1165,11 +1165,11 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>520537</v>
+        <v>520538</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>f972c07dbc579296ad8a1c8faaadf0c67943bb380e333121fab6f37b61c66031</t>
+          <t>28ab27d4343f0f6a158a360d1ceaffac4110e26d5a15771fd99492ee1f7b3498</t>
         </is>
       </c>
     </row>
@@ -1180,11 +1180,11 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>45570</v>
+        <v>46326</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>57538fa17db33a2cddc13bc5a9f910b1673f3181ce33919ca2d8a66ae38317af</t>
+          <t>d1a3a5b253c49e00fac97d632590e3a49477f05db294a0fea39fe5670c428352</t>
         </is>
       </c>
     </row>
@@ -1210,11 +1210,11 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>84790</v>
+        <v>84791</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1fb2c61017f90a2638871ce56ba7ba51ff8787abf224529202e0345b11336222</t>
+          <t>ca5d2c91ea2f9072d9829c85534dfc0ea59ac0d88ee962a7c6b7d1c85f9867ab</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>1222ce6fb9af8e7b25ac656042a3127b963182bce77172d2c0595ff885ba5ecb</t>
+          <t>f03c0ba2b0ccab34bbfb00340bba874b567eb31f98f07157aa77c04badae2db1</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>805142eb1fe1ced95bd7a2ae0152db33f430f5bc7e27b89c5d78c3756a689423</t>
+          <t>df5e7d013ecf2249fac140c6cd0ab98258ffe5e4897e0823e343f8834f6807ad</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>e430b9fc14647fcde8cc678f4e1a717332067b9da905c812c18a8564a6487331</t>
+          <t>57615be96f0bd1edd80accf81cdc638668eabe5ccd9adf59311b849a73191ccc</t>
         </is>
       </c>
     </row>

</xml_diff>